<commit_message>
Stop using examples in prompt (still use in search) + extract info from each examples one-by-one then combine
</commit_message>
<xml_diff>
--- a/eval_reports/pmid_41823034_eval_report_advp_like.xlsx
+++ b/eval_reports/pmid_41823034_eval_report_advp_like.xlsx
@@ -538,7 +538,7 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>depression + bipolar disorder + schizophrenia + alzheimers disease</t>
+          <t>bipolar disorder + schizophrenia + alzheimers disease + depression</t>
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
@@ -576,7 +576,7 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>depression + bipolar disorder + schizophrenia + alzheimers disease</t>
+          <t>bipolar disorder + schizophrenia + alzheimers disease + depression</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -614,7 +614,7 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>depression + bipolar disorder + schizophrenia + alzheimers disease</t>
+          <t>bipolar disorder + schizophrenia + alzheimers disease + depression</t>
         </is>
       </c>
       <c r="O4" t="inlineStr"/>
@@ -652,7 +652,7 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
-          <t>depression + bipolar disorder + schizophrenia + alzheimers disease</t>
+          <t>bipolar disorder + schizophrenia + alzheimers disease + depression</t>
         </is>
       </c>
       <c r="O5" t="inlineStr"/>
@@ -690,7 +690,7 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
-          <t>depression + bipolar disorder + schizophrenia + alzheimers disease</t>
+          <t>bipolar disorder + schizophrenia + alzheimers disease + depression</t>
         </is>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -728,7 +728,7 @@
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
-          <t>depression + bipolar disorder + schizophrenia + alzheimers disease</t>
+          <t>bipolar disorder + schizophrenia + alzheimers disease + depression</t>
         </is>
       </c>
       <c r="O7" t="inlineStr"/>
@@ -766,7 +766,7 @@
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
-          <t>depression + bipolar disorder + schizophrenia + alzheimers disease</t>
+          <t>bipolar disorder + schizophrenia + alzheimers disease + depression</t>
         </is>
       </c>
       <c r="O8" t="inlineStr"/>
@@ -804,7 +804,7 @@
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
-          <t>depression + bipolar disorder + schizophrenia + alzheimers disease</t>
+          <t>bipolar disorder + schizophrenia + alzheimers disease + depression</t>
         </is>
       </c>
       <c r="O9" t="inlineStr"/>
@@ -842,7 +842,7 @@
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
-          <t>depression + bipolar disorder + schizophrenia + alzheimers disease</t>
+          <t>bipolar disorder + schizophrenia + alzheimers disease + depression</t>
         </is>
       </c>
       <c r="O10" t="inlineStr"/>
@@ -880,7 +880,7 @@
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
-          <t>depression + bipolar disorder + schizophrenia + alzheimers disease</t>
+          <t>bipolar disorder + schizophrenia + alzheimers disease + depression</t>
         </is>
       </c>
       <c r="O11" t="inlineStr"/>
@@ -918,7 +918,7 @@
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
-          <t>depression + bipolar disorder + schizophrenia + alzheimers disease</t>
+          <t>bipolar disorder + schizophrenia + alzheimers disease + depression</t>
         </is>
       </c>
       <c r="O12" t="inlineStr"/>
@@ -956,7 +956,7 @@
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
-          <t>depression + bipolar disorder + schizophrenia + alzheimers disease</t>
+          <t>bipolar disorder + schizophrenia + alzheimers disease + depression</t>
         </is>
       </c>
       <c r="O13" t="inlineStr"/>
@@ -994,7 +994,7 @@
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
-          <t>depression + bipolar disorder + schizophrenia + alzheimers disease</t>
+          <t>bipolar disorder + schizophrenia + alzheimers disease + depression</t>
         </is>
       </c>
       <c r="O14" t="inlineStr"/>
@@ -1032,7 +1032,7 @@
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
-          <t>depression + bipolar disorder + schizophrenia + alzheimers disease</t>
+          <t>bipolar disorder + schizophrenia + alzheimers disease + depression</t>
         </is>
       </c>
       <c r="O15" t="inlineStr"/>
@@ -1070,7 +1070,7 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>depression + bipolar disorder + schizophrenia + alzheimers disease</t>
+          <t>bipolar disorder + schizophrenia + alzheimers disease + depression</t>
         </is>
       </c>
       <c r="O16" t="inlineStr"/>

</xml_diff>